<commit_message>
updated comments and motor calibration notes
</commit_message>
<xml_diff>
--- a/og/calibration results/2026-10-01-wavelength-vs-steps-vis/motor_calibration.xlsx
+++ b/og/calibration results/2026-10-01-wavelength-vs-steps-vis/motor_calibration.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andrew\Documents\aab_git\lab\arduino-bli-mono-controller\og\calibration results\2026-10-01-wavelength-vs-steps-vis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="e:\andrew\aab_git\lab\arduino-bli-mono-controller\og\calibration results\2026-10-01-wavelength-vs-steps-vis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{789410CF-8BDA-4E0C-B6E0-494647CEC8C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A0BB6D5-176C-4F0C-8FAC-84B86B56CB2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FDE96593-49B9-433C-9526-704AAE7475A3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FDE96593-49B9-433C-9526-704AAE7475A3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Steps_diff</t>
   </si>
@@ -53,7 +53,13 @@
     <t>calc'd</t>
   </si>
   <si>
-    <t>max</t>
+    <t>initial tests</t>
+  </si>
+  <si>
+    <t>set as home</t>
+  </si>
+  <si>
+    <t>set as steps_Max</t>
   </si>
 </sst>
 </file>
@@ -61,9 +67,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -74,6 +80,12 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -99,12 +111,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -301,10 +314,10 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$D$2:$D$19</c:f>
+              <c:f>Sheet1!$D$2:$D$4</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="18"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -319,10 +332,10 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$E$2:$E$19</c:f>
+              <c:f>Sheet1!$E$2:$E$4</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="18"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -1204,16 +1217,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>7620</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>407670</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>64770</xdr:rowOff>
+      <xdr:rowOff>45720</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>312420</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>64770</xdr:rowOff>
+      <xdr:colOff>102870</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1558,16 +1571,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DC04BB0-3A5B-4919-9E84-5D13CD47D85C}">
-  <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="8.88671875" style="2"/>
-    <col min="3" max="3" width="11.5546875" customWidth="1"/>
-    <col min="4" max="4" width="12.6640625" customWidth="1"/>
-    <col min="5" max="5" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19" customWidth="1"/>
+    <col min="2" max="2" width="8.85546875" style="2"/>
+    <col min="3" max="3" width="11.5703125" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
         <v>2</v>
       </c>
@@ -1581,7 +1595,10 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
       <c r="B2" s="2">
         <v>5328</v>
       </c>
@@ -1597,7 +1614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B3" s="2">
         <v>9008</v>
       </c>
@@ -1613,7 +1630,7 @@
         <v>-229.5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B4" s="2">
         <v>11568</v>
       </c>
@@ -1629,64 +1646,67 @@
         <v>-390</v>
       </c>
     </row>
-    <row r="5" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+    <row r="6" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="3">
-        <f>B$2-16*(C5-C$2)</f>
-        <v>8982.4</v>
-      </c>
-      <c r="C5" s="1">
-        <v>546.1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B6" s="3">
         <f>B$2-16*(C6-C$2)</f>
-        <v>8984</v>
+        <v>8982.4</v>
       </c>
       <c r="C6" s="1">
-        <v>546</v>
+        <v>546.1</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>6</v>
+      </c>
       <c r="B7" s="3">
         <f>B$2-16*(C7-C$2)</f>
-        <v>10747.2</v>
+        <v>8984</v>
       </c>
       <c r="C7" s="1">
-        <v>435.8</v>
+        <v>546</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B8" s="3">
         <f>B$2-16*(C8-C$2)</f>
-        <v>11880</v>
+        <v>10747.2</v>
       </c>
       <c r="C8" s="1">
-        <v>365</v>
+        <v>435.8</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B9" s="3">
         <f>B$2-16*(C9-C$2)</f>
+        <v>11880</v>
+      </c>
+      <c r="C9" s="1">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B10" s="3">
+        <f>B$2-16*(C10-C$2)</f>
         <v>13880</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C10" s="1">
         <v>240</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>5</v>
-      </c>
-      <c r="B10" s="2">
-        <v>16000</v>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" s="2">
+        <v>14000</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B12" s="4"/>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B13" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>